<commit_message>
Update reports 2026-09-17 10:07
</commit_message>
<xml_diff>
--- a/gex_pivot_levels_2026-09-17.xlsx
+++ b/gex_pivot_levels_2026-09-17.xlsx
@@ -676,12 +676,12 @@
       </c>
       <c r="D6" s="7" t="inlineStr">
         <is>
-          <t>-$3.60M</t>
+          <t>-$3.32M</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>+$4.63M</t>
+          <t>+$4.27M</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
@@ -870,12 +870,12 @@
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>+$1.91M</t>
+          <t>+$1.87M</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>+$11.12M</t>
+          <t>+$10.83M</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -961,12 +961,12 @@
       </c>
       <c r="D15" s="9" t="inlineStr">
         <is>
-          <t>+$5.03M</t>
+          <t>+$5.10M</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr">
         <is>
-          <t>+$12.62M</t>
+          <t>+$12.80M</t>
         </is>
       </c>
       <c r="F15" s="3" t="inlineStr">
@@ -1023,12 +1023,12 @@
       </c>
       <c r="D17" s="7" t="inlineStr">
         <is>
-          <t>-$151.19K</t>
+          <t>-$153.15K</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>+$7.68M</t>
+          <t>+$7.78M</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1056,12 +1056,12 @@
       </c>
       <c r="D18" s="9" t="inlineStr">
         <is>
-          <t>+$16.60M</t>
+          <t>+$17.02M</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>+$28.49M</t>
+          <t>+$29.20M</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
@@ -1089,12 +1089,12 @@
       </c>
       <c r="D19" s="8" t="inlineStr">
         <is>
-          <t>+$4.38M</t>
+          <t>+$4.49M</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>+$9.32M</t>
+          <t>+$9.55M</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
@@ -1122,12 +1122,12 @@
       </c>
       <c r="D20" s="9" t="inlineStr">
         <is>
-          <t>+$13.15M</t>
+          <t>+$13.62M</t>
         </is>
       </c>
       <c r="E20" s="3" t="inlineStr">
         <is>
-          <t>+$25.59M</t>
+          <t>+$26.50M</t>
         </is>
       </c>
       <c r="F20" s="3" t="inlineStr">
@@ -1188,12 +1188,12 @@
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>+$7.00M</t>
+          <t>+$7.33M</t>
         </is>
       </c>
       <c r="E22" s="6" t="inlineStr">
         <is>
-          <t>+$15.67M</t>
+          <t>+$16.42M</t>
         </is>
       </c>
       <c r="F22" s="6" t="inlineStr">
@@ -1217,12 +1217,12 @@
       </c>
       <c r="D23" s="4" t="inlineStr">
         <is>
-          <t>-$3.88M</t>
+          <t>-$4.00M</t>
         </is>
       </c>
       <c r="E23" s="3" t="inlineStr">
         <is>
-          <t>+$27.79M</t>
+          <t>+$28.69M</t>
         </is>
       </c>
       <c r="F23" s="3" t="inlineStr">
@@ -3365,12 +3365,12 @@
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>+$16.60M</t>
+          <t>+$17.02M</t>
         </is>
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>+$28.49M</t>
+          <t>+$29.20M</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -3403,12 +3403,12 @@
       </c>
       <c r="E4" s="4" t="inlineStr">
         <is>
-          <t>-$3.88M</t>
+          <t>-$4.00M</t>
         </is>
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>+$27.79M</t>
+          <t>+$28.69M</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -3441,12 +3441,12 @@
       </c>
       <c r="E5" s="9" t="inlineStr">
         <is>
-          <t>+$13.15M</t>
+          <t>+$13.62M</t>
         </is>
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>+$25.59M</t>
+          <t>+$26.50M</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -3627,12 +3627,12 @@
       </c>
       <c r="E10" s="8" t="inlineStr">
         <is>
-          <t>+$7.00M</t>
+          <t>+$7.33M</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>+$15.67M</t>
+          <t>+$16.42M</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
@@ -3737,12 +3737,12 @@
       </c>
       <c r="E13" s="9" t="inlineStr">
         <is>
-          <t>+$5.03M</t>
+          <t>+$5.10M</t>
         </is>
       </c>
       <c r="F13" s="3" t="inlineStr">
         <is>
-          <t>+$12.62M</t>
+          <t>+$12.80M</t>
         </is>
       </c>
       <c r="G13" s="3" t="inlineStr">
@@ -3869,28 +3869,28 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>ES</t>
+          <t>NQ</t>
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>7667.94</v>
+        <v>29518.07</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>7550</v>
+        <v>706</v>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E17" s="8" t="inlineStr">
-        <is>
-          <t>+$1.91M</t>
+          <t>QQQ</t>
+        </is>
+      </c>
+      <c r="E17" s="7" t="inlineStr">
+        <is>
+          <t>-$864.10K</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
         <is>
-          <t>+$11.12M</t>
+          <t>+$10.96M</t>
         </is>
       </c>
       <c r="G17" s="6" t="inlineStr">
@@ -3903,28 +3903,28 @@
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>NQ</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B18" s="5" t="n">
-        <v>29518.07</v>
+        <v>7667.94</v>
       </c>
       <c r="C18" s="5" t="n">
-        <v>706</v>
+        <v>7550</v>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>QQQ</t>
-        </is>
-      </c>
-      <c r="E18" s="7" t="inlineStr">
-        <is>
-          <t>-$864.10K</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>+$1.87M</t>
         </is>
       </c>
       <c r="F18" s="6" t="inlineStr">
         <is>
-          <t>+$10.96M</t>
+          <t>+$10.83M</t>
         </is>
       </c>
       <c r="G18" s="6" t="inlineStr">
@@ -4135,12 +4135,12 @@
       </c>
       <c r="E24" s="8" t="inlineStr">
         <is>
-          <t>+$4.38M</t>
+          <t>+$4.49M</t>
         </is>
       </c>
       <c r="F24" s="6" t="inlineStr">
         <is>
-          <t>+$9.32M</t>
+          <t>+$9.55M</t>
         </is>
       </c>
       <c r="G24" s="6" t="inlineStr">
@@ -4279,12 +4279,12 @@
       </c>
       <c r="E28" s="7" t="inlineStr">
         <is>
-          <t>-$151.19K</t>
+          <t>-$153.15K</t>
         </is>
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>+$7.68M</t>
+          <t>+$7.78M</t>
         </is>
       </c>
       <c r="G28" s="6" t="inlineStr">
@@ -4633,114 +4633,114 @@
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="6" t="inlineStr">
+      <c r="A38" s="3" t="inlineStr">
         <is>
           <t>ES</t>
         </is>
       </c>
-      <c r="B38" s="5" t="n">
-        <v>7617.94</v>
-      </c>
-      <c r="C38" s="5" t="n">
-        <v>7500</v>
-      </c>
-      <c r="D38" s="6" t="inlineStr">
-        <is>
-          <t>SPX</t>
-        </is>
-      </c>
-      <c r="E38" s="7" t="inlineStr">
-        <is>
-          <t>-$3.60M</t>
-        </is>
-      </c>
-      <c r="F38" s="6" t="inlineStr">
+      <c r="B38" s="2" t="n">
+        <v>7498.99</v>
+      </c>
+      <c r="C38" s="2" t="n">
+        <v>737</v>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>SPY</t>
+        </is>
+      </c>
+      <c r="E38" s="4" t="inlineStr">
+        <is>
+          <t>-$4.62M</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
         <is>
           <t>+$4.63M</t>
         </is>
       </c>
-      <c r="G38" s="6" t="inlineStr">
-        <is>
-          <t>Abs</t>
-        </is>
-      </c>
-      <c r="H38" s="6" t="inlineStr"/>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Both</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>valley</t>
+        </is>
+      </c>
     </row>
     <row r="39">
-      <c r="A39" s="3" t="inlineStr">
-        <is>
-          <t>ES</t>
-        </is>
-      </c>
-      <c r="B39" s="2" t="n">
-        <v>7498.99</v>
-      </c>
-      <c r="C39" s="2" t="n">
-        <v>737</v>
-      </c>
-      <c r="D39" s="3" t="inlineStr">
-        <is>
-          <t>SPY</t>
-        </is>
-      </c>
-      <c r="E39" s="4" t="inlineStr">
-        <is>
-          <t>-$4.62M</t>
-        </is>
-      </c>
-      <c r="F39" s="3" t="inlineStr">
-        <is>
-          <t>+$4.63M</t>
-        </is>
-      </c>
-      <c r="G39" s="3" t="inlineStr">
-        <is>
-          <t>Both</t>
-        </is>
-      </c>
-      <c r="H39" s="3" t="inlineStr">
-        <is>
-          <t>valley</t>
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>GC</t>
+        </is>
+      </c>
+      <c r="B39" s="5" t="n">
+        <v>4718.48</v>
+      </c>
+      <c r="C39" s="5" t="n">
+        <v>101</v>
+      </c>
+      <c r="D39" s="6" t="inlineStr">
+        <is>
+          <t>GDX</t>
+        </is>
+      </c>
+      <c r="E39" s="8" t="inlineStr">
+        <is>
+          <t>+$4.34M</t>
+        </is>
+      </c>
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>+$4.47M</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>Net</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>peak</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>GC</t>
+          <t>ES</t>
         </is>
       </c>
       <c r="B40" s="5" t="n">
-        <v>4718.48</v>
+        <v>7617.94</v>
       </c>
       <c r="C40" s="5" t="n">
-        <v>101</v>
+        <v>7500</v>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>GDX</t>
-        </is>
-      </c>
-      <c r="E40" s="8" t="inlineStr">
-        <is>
-          <t>+$4.34M</t>
+          <t>SPX</t>
+        </is>
+      </c>
+      <c r="E40" s="7" t="inlineStr">
+        <is>
+          <t>-$3.32M</t>
         </is>
       </c>
       <c r="F40" s="6" t="inlineStr">
         <is>
-          <t>+$4.47M</t>
+          <t>+$4.27M</t>
         </is>
       </c>
       <c r="G40" s="6" t="inlineStr">
         <is>
-          <t>Net</t>
-        </is>
-      </c>
-      <c r="H40" s="6" t="inlineStr">
-        <is>
-          <t>peak</t>
-        </is>
-      </c>
+          <t>Abs</t>
+        </is>
+      </c>
+      <c r="H40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="3" t="inlineStr">

</xml_diff>